<commit_message>
v2.1 review rounds 4-5: docs, review log, literature report
</commit_message>
<xml_diff>
--- a/literature-report-v21.xlsx
+++ b/literature-report-v21.xlsx
@@ -434,7 +434,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J8"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -779,12 +779,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Game texts (v21): lesson 8 step 1 and summary card, stage 8 end text, final end text; TEACHING_GUIDE v2.1 point 1</t>
+          <t>Game texts (v21): lesson 8 step 1 and summary card, stage 8 end text, final end text; TEACHING_GUIDE v2.1 point 1 and 'What to say' bullet 1</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>A real model learns how much each word should count for the question (its attention weights) and picks the next word from a blend of chances.</t>
+          <t>A real model learns how to decide how much each word counts (its attention).</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -794,17 +794,17 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Paraphrase</t>
+          <t>Quote</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>The output is computed as a weighted sum of the values, where the weight assigned to each value is computed by a compatibility function of the query with the corresponding key.</t>
+          <t>we found it beneficial to linearly project the queries, keys and values h times with different, learned linear projections</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>§3.2 (HTML, unpaginated)</t>
+          <t>§3.2.2 (HTML, unpaginated)</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr"/>
@@ -815,7 +815,53 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Plain-language paraphrase: 'how much each word counts' = the attention weights. 'Learns' refers to the trained model parameters; the excerpt itself does not say the weights are learned, so the game avoids more specific claims. 'Blend of chances' refers to next-word probabilities (taught in lesson 3).</t>
+          <t>'Learns how to decide' = the attention weights are computed for each input from learned projections. Simplified for beginners.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Game texts (v21): stage 8 end text ('the next word is picked from the chances (lesson 3)'), lesson 8 summary card; TEACHING_GUIDE v2.1 'What to say' bullet 1</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>A real model turns its output into chances (probabilities) for the next token.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Vaswani et al., 2017</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Quote</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>We also use the usual learned linear transformation and softmax function to convert the decoder output to predicted next-token probabilities.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>§3.4 (HTML, unpaginated)</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Verified against the full HTML text (excerpt saved)</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Links the toy's 'chances' (lesson 3) to the real model's next-token probabilities.</t>
         </is>
       </c>
     </row>

</xml_diff>